<commit_message>
feat: add color coded console markers
### Changed

- Add yellow `[ONLY]`, green `[COMPARE]`, and blue `[SAME]` console markers while keeping their message text in the terminal's default foreground for readability.
- Update examples to show also `Only in file1`/`Only in file2` situations
</commit_message>
<xml_diff>
--- a/examples/a.xlsx
+++ b/examples/a.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Dropbox\Work\godsdev-github\xlsx-compare\example\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Dropbox\Work\godsdev-github\xlsx-compare\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B075D173-5031-453A-B7FC-4EE3B86E66AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5930FA5B-1291-4B2E-AAA0-EA5157B964BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="7740" xr2:uid="{42AC03BA-AE0B-4E1D-9B7A-ED345BAA2529}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{42AC03BA-AE0B-4E1D-9B7A-ED345BAA2529}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="OnlyA" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -436,4 +437,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{110F2153-637E-427C-8F9A-E69A8C6F94F9}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>